<commit_message>
feat: update documentation and models to clarify DQA4 operational status and its impact on SVQ1 flow analysis also changed Costes_Vehiculos_UNIFICAR_SVQ1.xlsx data: small correction on number of vehicles and its data
</commit_message>
<xml_diff>
--- a/data/Costes_Vehiculos_UNIFICAR_SVQ1.xlsx
+++ b/data/Costes_Vehiculos_UNIFICAR_SVQ1.xlsx
@@ -94,12 +94,6 @@
     <t>26 VEHÍCULOS</t>
   </si>
   <si>
-    <t>19 furgonetas sin kms pero con dietas</t>
-  </si>
-  <si>
-    <t>19 VEHÍCULOS</t>
-  </si>
-  <si>
     <t>75 furgonetas con kms y dietas</t>
   </si>
   <si>
@@ -134,6 +128,12 @@
   </si>
   <si>
     <t>SOBRECOSTE ANUAL (€)</t>
+  </si>
+  <si>
+    <t>9 VEHÍCULOS</t>
+  </si>
+  <si>
+    <t>9 furgonetas sin kms pero con dietas</t>
   </si>
 </sst>
 </file>
@@ -142,7 +142,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -312,36 +312,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -350,8 +350,8 @@
     <xf numFmtId="44" fontId="8" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -679,23 +679,23 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="6" t="s">
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="R1" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="R1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
     </row>
     <row r="2" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -728,7 +728,7 @@
         <v>3</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="R4" s="3" t="s">
         <v>2</v>
@@ -737,145 +737,145 @@
         <v>3</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <f>SUM(B6,B21)</f>
         <v>61012.929999999993</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="7">
         <f>SUM(I6,I21)</f>
         <v>48370.929999999993</v>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="11">
         <f>I5*26</f>
         <v>1257644.1799999997</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="N5" s="8">
+      <c r="N5" s="7">
         <f>SUM(N6,N21)</f>
         <v>54739.729999999996</v>
       </c>
-      <c r="O5" s="12">
-        <f>N5*19</f>
-        <v>1040054.8699999999</v>
+      <c r="O5" s="11">
+        <f>N5*9</f>
+        <v>492657.56999999995</v>
       </c>
       <c r="R5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="S5" s="8">
+      <c r="S5" s="7">
         <f>SUM(S6,S21)</f>
         <v>61012.929999999993</v>
       </c>
-      <c r="T5" s="12">
+      <c r="T5" s="11">
         <f>S5*75</f>
         <v>4575969.7499999991</v>
       </c>
       <c r="W5" t="s">
-        <v>33</v>
-      </c>
-      <c r="X5" s="11">
+        <v>31</v>
+      </c>
+      <c r="X5" s="10">
         <f>SUM(J5,O5,T5)</f>
-        <v>6873668.7999999989</v>
+        <v>6326271.4999999981</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <f>SUM(B7,B13)</f>
         <v>57289.139999999992</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <f>SUM(I7,I13)</f>
         <v>44647.139999999992</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="10">
         <f t="shared" ref="J6:J21" si="0">I6*26</f>
         <v>1160825.6399999999</v>
       </c>
       <c r="M6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="N6" s="8">
+      <c r="N6" s="7">
         <f>SUM(N7,N13)</f>
         <v>51015.939999999995</v>
       </c>
-      <c r="O6" s="11">
-        <f t="shared" ref="O6:O21" si="1">N6*19</f>
-        <v>969302.85999999987</v>
+      <c r="O6" s="10">
+        <f t="shared" ref="O6:O21" si="1">N6*9</f>
+        <v>459143.45999999996</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="S6" s="8">
+      <c r="S6" s="7">
         <f>SUM(S7,S13)</f>
         <v>57289.139999999992</v>
       </c>
-      <c r="T6" s="11">
+      <c r="T6" s="10">
         <f t="shared" ref="T6:T21" si="2">S6*75</f>
         <v>4296685.4999999991</v>
       </c>
       <c r="W6" t="s">
-        <v>34</v>
-      </c>
-      <c r="X6" s="11">
-        <f>51*45000</f>
-        <v>2295000</v>
+        <v>32</v>
+      </c>
+      <c r="X6" s="10">
+        <f>61*45000</f>
+        <v>2745000</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <f>SUM(B8:B12)</f>
         <v>42116.469999999994</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="8">
         <f>SUM(I8:I12)</f>
         <v>42116.469999999994</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="10">
         <f t="shared" si="0"/>
         <v>1095028.2199999997</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="8">
         <f>SUM(N8:N12)</f>
         <v>42116.469999999994</v>
       </c>
-      <c r="O7" s="11">
+      <c r="O7" s="10">
         <f t="shared" si="1"/>
-        <v>800212.92999999993</v>
+        <v>379048.22999999992</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="S7" s="9">
+      <c r="S7" s="8">
         <f>SUM(S8:S12)</f>
         <v>42116.469999999994</v>
       </c>
-      <c r="T7" s="11">
+      <c r="T7" s="10">
         <f t="shared" si="2"/>
         <v>3158735.2499999995</v>
       </c>
@@ -884,81 +884,81 @@
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>2468.48</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="8">
         <v>2468.48</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="10">
         <f t="shared" si="0"/>
         <v>64180.480000000003</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="9">
+      <c r="N8" s="8">
         <v>2468.48</v>
       </c>
-      <c r="O8" s="11">
+      <c r="O8" s="10">
         <f t="shared" si="1"/>
-        <v>46901.120000000003</v>
+        <v>22216.32</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="S8" s="9">
+      <c r="S8" s="8">
         <v>2468.48</v>
       </c>
-      <c r="T8" s="11">
+      <c r="T8" s="10">
         <f t="shared" si="2"/>
         <v>185136</v>
       </c>
-      <c r="W8" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="X8" s="17">
+      <c r="W8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="X8" s="16">
         <f>SUM(X5:X6)</f>
-        <v>9168668.7999999989</v>
+        <v>9071271.4999999981</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>535.87</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="8">
         <v>535.87</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="10">
         <f t="shared" si="0"/>
         <v>13932.62</v>
       </c>
       <c r="M9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N9" s="9">
+      <c r="N9" s="8">
         <v>535.87</v>
       </c>
-      <c r="O9" s="11">
+      <c r="O9" s="10">
         <f t="shared" si="1"/>
-        <v>10181.530000000001</v>
+        <v>4822.83</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="S9" s="9">
+      <c r="S9" s="8">
         <v>535.87</v>
       </c>
-      <c r="T9" s="11">
+      <c r="T9" s="10">
         <f t="shared" si="2"/>
         <v>40190.25</v>
       </c>
@@ -967,36 +967,36 @@
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>33750.92</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="8">
         <v>33750.92</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="10">
         <f t="shared" si="0"/>
         <v>877523.91999999993</v>
       </c>
       <c r="M10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N10" s="9">
+      <c r="N10" s="8">
         <v>33750.92</v>
       </c>
-      <c r="O10" s="11">
+      <c r="O10" s="10">
         <f t="shared" si="1"/>
-        <v>641267.48</v>
+        <v>303758.27999999997</v>
       </c>
       <c r="R10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="S10" s="9">
+      <c r="S10" s="8">
         <v>33750.92</v>
       </c>
-      <c r="T10" s="11">
+      <c r="T10" s="10">
         <f t="shared" si="2"/>
         <v>2531319</v>
       </c>
@@ -1005,36 +1005,36 @@
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>4807.5</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="8">
         <v>4807.5</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="10">
         <f t="shared" si="0"/>
         <v>124995</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="N11" s="9">
+      <c r="N11" s="8">
         <v>4807.5</v>
       </c>
-      <c r="O11" s="11">
+      <c r="O11" s="10">
         <f t="shared" si="1"/>
-        <v>91342.5</v>
+        <v>43267.5</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="S11" s="9">
+      <c r="S11" s="8">
         <v>4807.5</v>
       </c>
-      <c r="T11" s="11">
+      <c r="T11" s="10">
         <f t="shared" si="2"/>
         <v>360562.5</v>
       </c>
@@ -1043,36 +1043,36 @@
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <v>553.70000000000005</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="7">
         <v>553.70000000000005</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="10">
         <f t="shared" si="0"/>
         <v>14396.2</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="N12" s="8">
+      <c r="N12" s="7">
         <v>553.70000000000005</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12" s="10">
         <f t="shared" si="1"/>
-        <v>10520.300000000001</v>
+        <v>4983.3</v>
       </c>
       <c r="R12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="S12" s="8">
+      <c r="S12" s="7">
         <v>553.70000000000005</v>
       </c>
-      <c r="T12" s="11">
+      <c r="T12" s="10">
         <f t="shared" si="2"/>
         <v>41527.5</v>
       </c>
@@ -1081,40 +1081,40 @@
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <f>SUM(B14:B19)</f>
         <v>15172.669999999998</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="9">
         <f>SUM(I14:I19)</f>
         <v>2530.67</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="10">
         <f t="shared" si="0"/>
         <v>65797.42</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N13" s="10">
+      <c r="N13" s="9">
         <f>SUM(N14:N19)</f>
         <v>8899.4700000000012</v>
       </c>
-      <c r="O13" s="11">
+      <c r="O13" s="10">
         <f t="shared" si="1"/>
-        <v>169089.93000000002</v>
+        <v>80095.23000000001</v>
       </c>
       <c r="R13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="S13" s="10">
+      <c r="S13" s="9">
         <f>SUM(S14:S19)</f>
         <v>15172.669999999998</v>
       </c>
-      <c r="T13" s="11">
+      <c r="T13" s="10">
         <f t="shared" si="2"/>
         <v>1137950.2499999998</v>
       </c>
@@ -1123,36 +1123,36 @@
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>6273.2</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="6">
         <v>0</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="6">
         <v>0</v>
       </c>
-      <c r="O14" s="11">
+      <c r="O14" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="S14" s="7">
+      <c r="S14" s="6">
         <v>6273.2</v>
       </c>
-      <c r="T14" s="11">
+      <c r="T14" s="10">
         <f t="shared" si="2"/>
         <v>470490</v>
       </c>
@@ -1161,36 +1161,36 @@
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="6">
         <v>292.77</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="6">
         <v>292.77</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="10">
         <f t="shared" si="0"/>
         <v>7612.0199999999995</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N15" s="7">
+      <c r="N15" s="6">
         <v>292.77</v>
       </c>
-      <c r="O15" s="11">
+      <c r="O15" s="10">
         <f t="shared" si="1"/>
-        <v>5562.6299999999992</v>
+        <v>2634.93</v>
       </c>
       <c r="R15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="S15" s="7">
+      <c r="S15" s="6">
         <v>292.77</v>
       </c>
-      <c r="T15" s="11">
+      <c r="T15" s="10">
         <f t="shared" si="2"/>
         <v>21957.75</v>
       </c>
@@ -1199,36 +1199,36 @@
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="6">
         <v>707.2</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="6">
         <v>707.2</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="10">
         <f t="shared" si="0"/>
         <v>18387.2</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N16" s="7">
+      <c r="N16" s="6">
         <v>707.2</v>
       </c>
-      <c r="O16" s="11">
+      <c r="O16" s="10">
         <f t="shared" si="1"/>
-        <v>13436.800000000001</v>
+        <v>6364.8</v>
       </c>
       <c r="R16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S16" s="7">
+      <c r="S16" s="6">
         <v>707.2</v>
       </c>
-      <c r="T16" s="11">
+      <c r="T16" s="10">
         <f t="shared" si="2"/>
         <v>53040</v>
       </c>
@@ -1237,36 +1237,36 @@
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="6">
         <v>551.04999999999995</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="6">
         <v>551.04999999999995</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="10">
         <f t="shared" si="0"/>
         <v>14327.3</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="6">
         <v>551.04999999999995</v>
       </c>
-      <c r="O17" s="11">
+      <c r="O17" s="10">
         <f t="shared" si="1"/>
-        <v>10469.949999999999</v>
+        <v>4959.45</v>
       </c>
       <c r="R17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S17" s="7">
+      <c r="S17" s="6">
         <v>551.04999999999995</v>
       </c>
-      <c r="T17" s="11">
+      <c r="T17" s="10">
         <f t="shared" si="2"/>
         <v>41328.75</v>
       </c>
@@ -1275,36 +1275,36 @@
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="6">
         <v>979.65</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="6">
         <v>979.65</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="10">
         <f t="shared" si="0"/>
         <v>25470.899999999998</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="7">
+      <c r="N18" s="6">
         <v>979.65</v>
       </c>
-      <c r="O18" s="11">
+      <c r="O18" s="10">
         <f t="shared" si="1"/>
-        <v>18613.349999999999</v>
+        <v>8816.85</v>
       </c>
       <c r="R18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S18" s="7">
+      <c r="S18" s="6">
         <v>979.65</v>
       </c>
-      <c r="T18" s="11">
+      <c r="T18" s="10">
         <f t="shared" si="2"/>
         <v>73473.75</v>
       </c>
@@ -1313,36 +1313,36 @@
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="6">
         <v>6368.8</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="6">
         <v>0</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="6">
         <v>6368.8</v>
       </c>
-      <c r="O19" s="11">
+      <c r="O19" s="10">
         <f t="shared" si="1"/>
-        <v>121007.2</v>
+        <v>57319.200000000004</v>
       </c>
       <c r="R19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S19" s="7">
+      <c r="S19" s="6">
         <v>6368.8</v>
       </c>
-      <c r="T19" s="11">
+      <c r="T19" s="10">
         <f t="shared" si="2"/>
         <v>477660</v>
       </c>
@@ -1351,36 +1351,36 @@
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="7">
         <v>0</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="7">
         <v>0</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N20" s="8">
+      <c r="N20" s="7">
         <v>0</v>
       </c>
-      <c r="O20" s="11">
+      <c r="O20" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="S20" s="8">
+      <c r="S20" s="7">
         <v>0</v>
       </c>
-      <c r="T20" s="11">
+      <c r="T20" s="10">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -1389,74 +1389,74 @@
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="7">
         <v>3723.79</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="7">
         <v>3723.79</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="10">
         <f t="shared" si="0"/>
         <v>96818.54</v>
       </c>
       <c r="M21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N21" s="8">
+      <c r="N21" s="7">
         <v>3723.79</v>
       </c>
-      <c r="O21" s="11">
+      <c r="O21" s="10">
         <f t="shared" si="1"/>
-        <v>70752.009999999995</v>
+        <v>33514.11</v>
       </c>
       <c r="R21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="S21" s="8">
+      <c r="S21" s="7">
         <v>3723.79</v>
       </c>
-      <c r="T21" s="11">
+      <c r="T21" s="10">
         <f t="shared" si="2"/>
         <v>279284.25</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W22" s="22" t="s">
-        <v>37</v>
+      <c r="W22" s="17" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="W24" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="X24" s="19">
+      <c r="W24" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="X24" s="18">
         <f>SUM(X8,S29)/10^6</f>
-        <v>10.162412239999998</v>
+        <v>10.065014939999998</v>
       </c>
     </row>
     <row r="25" spans="1:27" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W25" s="18"/>
-      <c r="X25" s="19"/>
+      <c r="W25" s="19"/>
+      <c r="X25" s="18"/>
     </row>
     <row r="26" spans="1:27" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I26" s="6"/>
+      <c r="H26" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="I26" s="22"/>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="Z27" s="20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AA27" s="21">
         <f>(X24-X30)*10^6</f>
@@ -1483,10 +1483,10 @@
         <v>3</v>
       </c>
       <c r="O28" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="W28" s="22" t="s">
-        <v>38</v>
+        <v>29</v>
+      </c>
+      <c r="W28" s="17" t="s">
+        <v>36</v>
       </c>
       <c r="Z28" s="20"/>
       <c r="AA28" s="21"/>
@@ -1495,32 +1495,32 @@
       <c r="A29" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="7">
         <f>SUM(B30,B45)</f>
         <v>147422.31999999998</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I29" s="15">
+      <c r="I29" s="14">
         <f>SUM(I30,I45)</f>
         <v>147422.31999999998</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="N29" s="8">
+      <c r="N29" s="7">
         <f>SUM(N30,N45)</f>
         <v>141053.51999999999</v>
       </c>
-      <c r="O29" s="12">
+      <c r="O29" s="11">
         <f>N29*6</f>
         <v>846321.11999999988</v>
       </c>
-      <c r="R29" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="S29" s="17">
+      <c r="R29" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="S29" s="16">
         <f>SUM(I29,O29)</f>
         <v>993743.43999999983</v>
       </c>
@@ -1529,85 +1529,85 @@
       <c r="A30" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="7">
         <f>SUM(B31,B37)</f>
         <v>137725.15999999997</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="7">
         <f>SUM(I31,I37)</f>
         <v>137725.15999999997</v>
       </c>
       <c r="M30" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="N30" s="8">
+      <c r="N30" s="7">
         <f>SUM(N31,N37)</f>
         <v>131356.35999999999</v>
       </c>
-      <c r="O30" s="11">
+      <c r="O30" s="10">
         <f t="shared" ref="O30:O45" si="3">N30*6</f>
         <v>788138.15999999992</v>
       </c>
-      <c r="W30" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="X30" s="19">
+      <c r="W30" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="X30" s="18">
         <f>X24-(S5*2)/10^6</f>
-        <v>10.040386379999998</v>
+        <v>9.9429890799999967</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="8">
         <f>SUM(B32:B36)</f>
         <v>69147.03</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I31" s="9">
+      <c r="I31" s="8">
         <f>SUM(I32:I36)</f>
         <v>69147.03</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="N31" s="9">
+      <c r="N31" s="8">
         <f>SUM(N32:N36)</f>
         <v>69147.03</v>
       </c>
-      <c r="O31" s="11">
+      <c r="O31" s="10">
         <f t="shared" si="3"/>
         <v>414882.18</v>
       </c>
-      <c r="W31" s="18"/>
-      <c r="X31" s="19"/>
+      <c r="W31" s="19"/>
+      <c r="X31" s="18"/>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <v>18111.689999999999</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I32" s="9">
+      <c r="I32" s="8">
         <v>18111.689999999999</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="N32" s="9">
+      <c r="N32" s="8">
         <v>18111.689999999999</v>
       </c>
-      <c r="O32" s="11">
+      <c r="O32" s="10">
         <f t="shared" si="3"/>
         <v>108670.13999999998</v>
       </c>
@@ -1616,22 +1616,22 @@
       <c r="A33" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="8">
         <v>4254.0600000000004</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I33" s="9">
+      <c r="I33" s="8">
         <v>4254.0600000000004</v>
       </c>
       <c r="M33" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N33" s="9">
+      <c r="N33" s="8">
         <v>4254.0600000000004</v>
       </c>
-      <c r="O33" s="11">
+      <c r="O33" s="10">
         <f t="shared" si="3"/>
         <v>25524.36</v>
       </c>
@@ -1640,22 +1640,22 @@
       <c r="A34" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="8">
         <v>37501.03</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I34" s="9">
+      <c r="I34" s="8">
         <v>37501.03</v>
       </c>
       <c r="M34" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N34" s="9">
+      <c r="N34" s="8">
         <v>37501.03</v>
       </c>
-      <c r="O34" s="11">
+      <c r="O34" s="10">
         <f t="shared" si="3"/>
         <v>225006.18</v>
       </c>
@@ -1664,22 +1664,22 @@
       <c r="A35" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>8335.76</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I35" s="9">
+      <c r="I35" s="8">
         <v>8335.76</v>
       </c>
       <c r="M35" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="N35" s="9">
+      <c r="N35" s="8">
         <v>8335.76</v>
       </c>
-      <c r="O35" s="11">
+      <c r="O35" s="10">
         <f t="shared" si="3"/>
         <v>50014.559999999998</v>
       </c>
@@ -1688,22 +1688,22 @@
       <c r="A36" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="9">
         <v>944.49</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I36" s="10">
+      <c r="I36" s="9">
         <v>944.49</v>
       </c>
       <c r="M36" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N36" s="10">
+      <c r="N36" s="9">
         <v>944.49</v>
       </c>
-      <c r="O36" s="11">
+      <c r="O36" s="10">
         <f t="shared" si="3"/>
         <v>5666.9400000000005</v>
       </c>
@@ -1712,25 +1712,25 @@
       <c r="A37" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="7">
         <f>SUM(B38:B44)</f>
         <v>68578.12999999999</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I37" s="8">
+      <c r="I37" s="7">
         <f>SUM(I38:I44)</f>
         <v>68578.12999999999</v>
       </c>
       <c r="M37" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N37" s="8">
+      <c r="N37" s="7">
         <f>SUM(N38:N44)</f>
         <v>62209.329999999994</v>
       </c>
-      <c r="O37" s="11">
+      <c r="O37" s="10">
         <f t="shared" si="3"/>
         <v>373255.98</v>
       </c>
@@ -1739,22 +1739,22 @@
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>43763.65</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I38" s="9">
+      <c r="I38" s="8">
         <v>43763.65</v>
       </c>
       <c r="M38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N38" s="9">
+      <c r="N38" s="8">
         <v>43763.65</v>
       </c>
-      <c r="O38" s="11">
+      <c r="O38" s="10">
         <f t="shared" si="3"/>
         <v>262581.90000000002</v>
       </c>
@@ -1763,22 +1763,22 @@
       <c r="A39" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="8">
         <v>2138.4299999999998</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I39" s="9">
+      <c r="I39" s="8">
         <v>2138.4299999999998</v>
       </c>
       <c r="M39" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N39" s="9">
+      <c r="N39" s="8">
         <v>2138.4299999999998</v>
       </c>
-      <c r="O39" s="11">
+      <c r="O39" s="10">
         <f t="shared" si="3"/>
         <v>12830.579999999998</v>
       </c>
@@ -1787,22 +1787,22 @@
       <c r="A40" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>6997.73</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I40" s="9">
+      <c r="I40" s="8">
         <v>6997.73</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N40" s="9">
+      <c r="N40" s="8">
         <v>6997.73</v>
       </c>
-      <c r="O40" s="11">
+      <c r="O40" s="10">
         <f t="shared" si="3"/>
         <v>41986.38</v>
       </c>
@@ -1811,22 +1811,22 @@
       <c r="A41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="8">
         <v>2332.6799999999998</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I41" s="9">
+      <c r="I41" s="8">
         <v>2332.6799999999998</v>
       </c>
       <c r="M41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N41" s="9">
+      <c r="N41" s="8">
         <v>2332.6799999999998</v>
       </c>
-      <c r="O41" s="11">
+      <c r="O41" s="10">
         <f t="shared" si="3"/>
         <v>13996.079999999998</v>
       </c>
@@ -1835,22 +1835,22 @@
       <c r="A42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="8">
         <v>4591.92</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I42" s="9">
+      <c r="I42" s="8">
         <v>4591.92</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N42" s="9">
+      <c r="N42" s="8">
         <v>4591.92</v>
       </c>
-      <c r="O42" s="11">
+      <c r="O42" s="10">
         <f t="shared" si="3"/>
         <v>27551.52</v>
       </c>
@@ -1859,22 +1859,22 @@
       <c r="A43" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B43" s="14">
+      <c r="B43" s="13">
         <v>6368.8</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I43" s="7">
+      <c r="I43" s="6">
         <v>6368.8</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="N43" s="9">
+      <c r="N43" s="8">
         <v>0</v>
       </c>
-      <c r="O43" s="11">
+      <c r="O43" s="10">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1883,22 +1883,22 @@
       <c r="A44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>2384.92</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I44" s="9">
+      <c r="I44" s="8">
         <v>2384.92</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N44" s="9">
+      <c r="N44" s="8">
         <v>2384.92</v>
       </c>
-      <c r="O44" s="11">
+      <c r="O44" s="10">
         <f t="shared" si="3"/>
         <v>14309.52</v>
       </c>
@@ -1907,38 +1907,38 @@
       <c r="A45" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="7">
         <v>9697.16</v>
       </c>
       <c r="H45" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I45" s="8">
+      <c r="I45" s="7">
         <v>9697.16</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N45" s="8">
+      <c r="N45" s="7">
         <v>9697.16</v>
       </c>
-      <c r="O45" s="11">
+      <c r="O45" s="10">
         <f t="shared" si="3"/>
         <v>58182.96</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="R1:T1"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="W24:W25"/>
     <mergeCell ref="X24:X25"/>
     <mergeCell ref="W30:W31"/>
     <mergeCell ref="X30:X31"/>
     <mergeCell ref="Z27:Z28"/>
     <mergeCell ref="AA27:AA28"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="R1:T1"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="W24:W25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>